<commit_message>
final: annotated DXF outputs with stage9 fixes
</commit_message>
<xml_diff>
--- a/焊缝统计_auto.xlsx
+++ b/焊缝统计_auto.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焊缝统计" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="异常报告" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="抽检清单" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="焊缝统计" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="异常报告" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="抽检清单" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17052,10 +17052,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>461</v>
+        <v>220</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
@@ -17065,7 +17065,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>p53</t>
+          <t>p118</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -17110,14 +17110,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
@@ -17164,12 +17164,12 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>BE018</t>
+          <t>p52</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>p52</t>
+          <t>p53</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -17179,12 +17179,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -17194,7 +17194,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -17263,7 +17263,7 @@
         <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>140</v>
+        <v>39</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
@@ -17340,14 +17340,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D8" t="n">
-        <v>445</v>
+        <v>220</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
@@ -17357,7 +17357,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>p175</t>
+          <t>p118</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -17402,14 +17402,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D9" t="n">
-        <v>300</v>
+        <v>220</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
@@ -17456,7 +17456,7 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>BE020</t>
+          <t>p175</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -17471,12 +17471,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -17486,14 +17486,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>7</v>
       </c>
       <c r="D11" t="n">
-        <v>39</v>
+        <v>140</v>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
@@ -17528,19 +17528,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>140</v>
+        <v>39</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>p175</t>
+          <t>BE020</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -17555,12 +17555,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -17636,14 +17636,13 @@
           <t>Above</t>
         </is>
       </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
       <c r="D14" t="n">
-        <v>250</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>PL14mm</t>
-        </is>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>BE021</t>
@@ -17666,7 +17665,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -17676,7 +17675,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -17718,7 +17717,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -17763,14 +17762,13 @@
           <t>Above</t>
         </is>
       </c>
+      <c r="C17" t="n">
+        <v>12</v>
+      </c>
       <c r="D17" t="n">
-        <v>140</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>PL10mm</t>
-        </is>
-      </c>
+        <v>533.9</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>BE022</t>
@@ -17778,7 +17776,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>p200</t>
+          <t>p19</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -17793,7 +17791,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>FW</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -17823,16 +17821,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Below</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>6</v>
+          <t>Above</t>
+        </is>
       </c>
       <c r="D18" t="n">
-        <v>200</v>
-      </c>
-      <c r="E18" t="inlineStr"/>
+        <v>140</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>PL10mm</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>BE022</t>
@@ -17840,7 +17839,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>p26</t>
+          <t>p200</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -17855,7 +17854,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -17868,21 +17867,22 @@
           <t>Above</t>
         </is>
       </c>
-      <c r="C19" t="n">
-        <v>7</v>
-      </c>
       <c r="D19" t="n">
         <v>140</v>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>PL10mm</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>p18</t>
+          <t>BE022</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>p19</t>
+          <t>p200</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -17892,12 +17892,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -17919,12 +17919,12 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>BE022</t>
+          <t>p18</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>p18</t>
+          <t>p19</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -17934,12 +17934,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -17949,16 +17949,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Below</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>7</v>
+          <t>Above</t>
+        </is>
       </c>
       <c r="D21" t="n">
-        <v>29</v>
-      </c>
-      <c r="E21" t="inlineStr"/>
+        <v>140</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>PL10mm</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>BE022</t>
@@ -17966,7 +17967,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>p18</t>
+          <t>p200</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -17981,7 +17982,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -17991,14 +17992,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D22" t="n">
-        <v>140</v>
+        <v>440</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
@@ -18008,7 +18009,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>p48</t>
+          <t>p43</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -18099,7 +18100,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>438.9</v>
+        <v>140</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -18150,14 +18151,14 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
+          <t>BE023</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
           <t>p42</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>p43</t>
-        </is>
-      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>361-RC3210-S-01-BE023</t>
@@ -18165,12 +18166,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -18180,14 +18181,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>6</v>
       </c>
       <c r="D26" t="n">
-        <v>150</v>
+        <v>232</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
@@ -18197,7 +18198,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>p33</t>
+          <t>p83</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -18242,14 +18243,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>6</v>
       </c>
       <c r="D27" t="n">
-        <v>232</v>
+        <v>150</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
@@ -18259,7 +18260,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>p33</t>
+          <t>p83</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -18291,7 +18292,7 @@
         <v>6</v>
       </c>
       <c r="D28" t="n">
-        <v>150</v>
+        <v>232</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
@@ -18333,7 +18334,7 @@
         <v>7</v>
       </c>
       <c r="D29" t="n">
-        <v>172</v>
+        <v>220</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
@@ -18343,7 +18344,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>p47</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -18395,7 +18396,7 @@
         <v>7</v>
       </c>
       <c r="D30" t="n">
-        <v>60</v>
+        <v>220</v>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
@@ -18405,7 +18406,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>p126</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -18437,7 +18438,7 @@
         <v>7</v>
       </c>
       <c r="D31" t="n">
-        <v>220</v>
+        <v>115</v>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
@@ -18447,7 +18448,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>p125</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -18479,7 +18480,7 @@
         <v>7</v>
       </c>
       <c r="D32" t="n">
-        <v>220</v>
+        <v>115</v>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
@@ -18489,7 +18490,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>p125</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -18514,14 +18515,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D33" t="n">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
@@ -18531,7 +18532,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>p125</t>
+          <t>p126</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -18556,17 +18557,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Above</t>
-        </is>
+          <t>Below</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>7</v>
       </c>
       <c r="D34" t="n">
         <v>220</v>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>PL9mm</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>CO007</t>
@@ -18574,7 +18574,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>p124</t>
+          <t>p125</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -18589,7 +18589,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -18602,14 +18602,13 @@
           <t>Above</t>
         </is>
       </c>
+      <c r="C35" t="n">
+        <v>7</v>
+      </c>
       <c r="D35" t="n">
-        <v>116</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>PL9mm</t>
-        </is>
-      </c>
+        <v>313</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>CO007</t>
@@ -18617,7 +18616,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>p124</t>
+          <t>p100</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -18632,7 +18631,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -18642,24 +18641,24 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C36" t="n">
         <v>7</v>
       </c>
       <c r="D36" t="n">
-        <v>60</v>
+        <v>90.5</v>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>CO007</t>
+          <t>p100</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>p127</t>
+          <t>p124</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -18669,12 +18668,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -18726,14 +18725,14 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>7</v>
       </c>
       <c r="D38" t="n">
-        <v>250</v>
+        <v>115</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
@@ -18743,7 +18742,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>p92</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -18795,17 +18794,17 @@
         <v>7</v>
       </c>
       <c r="D39" t="n">
-        <v>115</v>
+        <v>90.5</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>CO008</t>
+          <t>p102</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>p101</t>
+          <t>p126</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -18815,12 +18814,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -18834,10 +18833,10 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D40" t="n">
-        <v>115</v>
+        <v>220</v>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
@@ -18872,16 +18871,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Below</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>9</v>
+          <t>Above</t>
+        </is>
       </c>
       <c r="D41" t="n">
-        <v>115</v>
-      </c>
-      <c r="E41" t="inlineStr"/>
+        <v>116</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>PL9mm</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>CO008</t>
@@ -18889,7 +18889,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>p125</t>
+          <t>p124</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -18904,7 +18904,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -18917,14 +18917,13 @@
           <t>Above</t>
         </is>
       </c>
+      <c r="C42" t="n">
+        <v>7</v>
+      </c>
       <c r="D42" t="n">
-        <v>116</v>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>PL9mm</t>
-        </is>
-      </c>
+        <v>90.5</v>
+      </c>
+      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>CO008</t>
@@ -18932,7 +18931,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>p124</t>
+          <t>p127</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -18947,7 +18946,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -18964,7 +18963,7 @@
         <v>7</v>
       </c>
       <c r="D43" t="n">
-        <v>90.5</v>
+        <v>60</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
@@ -18999,24 +18998,24 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>7</v>
       </c>
       <c r="D44" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>CO008</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>p127</t>
+          <t>p102</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -19026,12 +19025,12 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -19041,7 +19040,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -19053,7 +19052,7 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>CO008</t>
+          <t>p102</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -19068,12 +19067,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -19125,7 +19124,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -19187,14 +19186,14 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C48" t="n">
         <v>16</v>
       </c>
       <c r="D48" t="n">
-        <v>158</v>
+        <v>120</v>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
@@ -19204,7 +19203,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>p7</t>
+          <t>p16</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -19278,12 +19277,12 @@
         <v>16</v>
       </c>
       <c r="D50" t="n">
-        <v>158</v>
+        <v>405</v>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>p15</t>
+          <t>CO009</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -19298,12 +19297,12 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -19317,10 +19316,10 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D51" t="n">
-        <v>38</v>
+        <v>164.5</v>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
@@ -19330,7 +19329,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>p17</t>
+          <t>p144</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -19355,24 +19354,24 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D52" t="n">
-        <v>164.5</v>
+        <v>400</v>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>CO009</t>
+          <t>p16</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>p144</t>
+          <t>p7</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -19382,12 +19381,12 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -19397,14 +19396,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>12</v>
       </c>
       <c r="D53" t="n">
-        <v>110</v>
+        <v>200</v>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
@@ -19414,7 +19413,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>p194</t>
+          <t>p195</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -19459,14 +19458,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D54" t="n">
-        <v>200</v>
+        <v>262</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
@@ -19476,7 +19475,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>p195</t>
+          <t>p169</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -19501,14 +19500,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C55" t="n">
         <v>10</v>
       </c>
       <c r="D55" t="n">
-        <v>350</v>
+        <v>262</v>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
@@ -19543,14 +19542,14 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D56" t="n">
-        <v>262</v>
+        <v>139</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
@@ -19560,7 +19559,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>p169</t>
+          <t>p184</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -19588,14 +19587,13 @@
           <t>Above</t>
         </is>
       </c>
+      <c r="C57" t="n">
+        <v>9</v>
+      </c>
       <c r="D57" t="n">
         <v>139</v>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>PL12mm</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>CO010</t>
@@ -19603,7 +19601,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>p184</t>
+          <t>p185</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -19618,7 +19616,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -19632,7 +19630,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D58" t="n">
         <v>139</v>
@@ -19645,7 +19643,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>p185</t>
+          <t>p194</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -19670,11 +19668,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D59" t="n">
         <v>139</v>
@@ -19687,7 +19685,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>p194</t>
+          <t>p196</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -19712,14 +19710,14 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C60" t="n">
         <v>12</v>
       </c>
       <c r="D60" t="n">
-        <v>139</v>
+        <v>110</v>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
@@ -19729,7 +19727,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>p194</t>
+          <t>p197</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -19761,7 +19759,7 @@
         <v>12</v>
       </c>
       <c r="D61" t="n">
-        <v>139</v>
+        <v>110</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
@@ -19800,7 +19798,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D62" t="n">
         <v>139</v>
@@ -19813,7 +19811,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>p199</t>
+          <t>p197</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -19841,13 +19839,14 @@
           <t>Above</t>
         </is>
       </c>
-      <c r="C63" t="n">
-        <v>7</v>
-      </c>
       <c r="D63" t="n">
-        <v>139</v>
-      </c>
-      <c r="E63" t="inlineStr"/>
+        <v>260</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>PL12mm</t>
+        </is>
+      </c>
       <c r="F63" t="inlineStr">
         <is>
           <t>CO010</t>
@@ -19855,7 +19854,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>p199</t>
+          <t>p198</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -19870,7 +19869,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -19922,7 +19921,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -19971,7 +19970,7 @@
         <v>7</v>
       </c>
       <c r="D66" t="n">
-        <v>139</v>
+        <v>260</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
@@ -20013,7 +20012,7 @@
         <v>7</v>
       </c>
       <c r="D67" t="n">
-        <v>139</v>
+        <v>260</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
@@ -20052,7 +20051,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D68" t="n">
         <v>139</v>
@@ -20065,7 +20064,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>p207</t>
+          <t>p202</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -20178,10 +20177,10 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D71" t="n">
-        <v>260</v>
+        <v>139</v>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
@@ -20191,7 +20190,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>p207</t>
+          <t>p212</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -20216,24 +20215,24 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C72" t="n">
         <v>12</v>
       </c>
       <c r="D72" t="n">
-        <v>139</v>
+        <v>90</v>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>CO010</t>
+          <t>sp23</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>p212</t>
+          <t>p183</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -20243,12 +20242,12 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -20258,24 +20257,24 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C73" t="n">
         <v>12</v>
       </c>
       <c r="D73" t="n">
-        <v>139</v>
+        <v>90</v>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>CO010</t>
+          <t>sp23</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>p212</t>
+          <t>p183</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -20285,12 +20284,12 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -20300,24 +20299,24 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C74" t="n">
         <v>12</v>
       </c>
       <c r="D74" t="n">
-        <v>139</v>
+        <v>90</v>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>CO010</t>
+          <t>p182</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>p212</t>
+          <t>p183</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -20327,12 +20326,12 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -20354,7 +20353,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>sp23</t>
+          <t>p182</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -20384,7 +20383,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -20396,7 +20395,7 @@
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>sp23</t>
+          <t>p182</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -20426,7 +20425,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -20438,7 +20437,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>sp23</t>
+          <t>p182</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -20480,7 +20479,7 @@
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>sp23</t>
+          <t>p182</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -20522,7 +20521,7 @@
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>sp23</t>
+          <t>p182</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -20552,24 +20551,24 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D80" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>sp23</t>
+          <t>p195</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>p183</t>
+          <t>p196</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -20601,17 +20600,17 @@
         <v>12</v>
       </c>
       <c r="D81" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>p182</t>
+          <t>p195</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>p183</t>
+          <t>p212</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -20636,25 +20635,24 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Above</t>
-        </is>
+          <t>Below</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>12</v>
       </c>
       <c r="D82" t="n">
-        <v>324</v>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>PL10mm</t>
-        </is>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>p194</t>
+          <t>p195</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>p195</t>
+          <t>p212</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -20669,7 +20667,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -20679,7 +20677,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C83" t="n">

</xml_diff>

<commit_message>
Balance weld label layout: half-zone, short leaders, inner frame
Restore short-first leader search and tighten quadrant fallback without cross_ok. Add inner-frame enforcement, WM avoidance, Y-slot stagger, and Part-bottom downward bias using Part-only bbox so other views keep normal orientation.

Regenerate annotated DXF/PDF outputs and weld statistics spreadsheet.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/焊缝统计_auto.xlsx
+++ b/焊缝统计_auto.xlsx
@@ -17048,14 +17048,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D2" t="n">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
@@ -17114,10 +17114,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>300</v>
+        <v>140</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
@@ -17127,7 +17127,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>p118</t>
+          <t>p52</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -17152,26 +17152,26 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>7</v>
       </c>
       <c r="D4" t="n">
-        <v>140</v>
+        <v>39</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
+          <t>BE018</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>p52</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>p53</t>
-        </is>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>361-RC3210-S-01-BE018</t>
@@ -17179,12 +17179,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -17194,14 +17194,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>12</v>
       </c>
       <c r="D5" t="n">
-        <v>300</v>
+        <v>429</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
@@ -17211,7 +17211,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>p118</t>
+          <t>p176</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -17256,14 +17256,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>39</v>
+        <v>220</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
@@ -17273,7 +17273,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>p52</t>
+          <t>p118</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -17298,19 +17298,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>39</v>
+        <v>140</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>BE019</t>
+          <t>p176</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -17325,12 +17325,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -17344,10 +17344,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D8" t="n">
-        <v>220</v>
+        <v>445</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
@@ -17357,7 +17357,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>p118</t>
+          <t>p175</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -17406,10 +17406,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D9" t="n">
-        <v>220</v>
+        <v>445</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
@@ -17419,7 +17419,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>p118</t>
+          <t>p175</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -17448,20 +17448,20 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D10" t="n">
-        <v>140</v>
+        <v>300</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>p175</t>
+          <t>BE020</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>p52</t>
+          <t>p118</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -17471,12 +17471,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -17498,7 +17498,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>BE020</t>
+          <t>p175</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -17513,12 +17513,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -17528,19 +17528,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>39</v>
+        <v>140</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>BE020</t>
+          <t>p175</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -17555,12 +17555,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -17570,17 +17570,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Above</t>
-        </is>
+          <t>Below</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
       </c>
       <c r="D13" t="n">
         <v>250</v>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>PL14mm</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>BE021</t>
@@ -17603,7 +17602,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>FW</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -17633,14 +17632,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D14" t="n">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
@@ -17650,7 +17649,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>p122</t>
+          <t>p123</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -17675,24 +17674,24 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>250</v>
+        <v>60</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>BE021</t>
+          <t>p122</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>p122</t>
+          <t>p123</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -17702,12 +17701,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -17724,12 +17723,12 @@
         <v>8</v>
       </c>
       <c r="D16" t="n">
-        <v>155</v>
+        <v>60</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>BE021</t>
+          <t>p122</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -17744,12 +17743,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -17762,13 +17761,14 @@
           <t>Above</t>
         </is>
       </c>
-      <c r="C17" t="n">
-        <v>12</v>
-      </c>
       <c r="D17" t="n">
-        <v>533.9</v>
-      </c>
-      <c r="E17" t="inlineStr"/>
+        <v>140</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PL10mm</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>BE022</t>
@@ -17776,7 +17776,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>p19</t>
+          <t>p200</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -17791,7 +17791,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -17824,22 +17824,21 @@
           <t>Above</t>
         </is>
       </c>
+      <c r="C18" t="n">
+        <v>7</v>
+      </c>
       <c r="D18" t="n">
         <v>140</v>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>PL10mm</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>BE022</t>
+          <t>p18</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>p200</t>
+          <t>p19</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -17849,12 +17848,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -17864,17 +17863,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Above</t>
-        </is>
+          <t>Below</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>7</v>
       </c>
       <c r="D19" t="n">
-        <v>140</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>PL10mm</t>
-        </is>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>BE022</t>
@@ -17882,7 +17880,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>p200</t>
+          <t>p18</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -17897,7 +17895,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -17907,26 +17905,26 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C20" t="n">
         <v>7</v>
       </c>
       <c r="D20" t="n">
-        <v>140</v>
+        <v>29</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
+          <t>BE022</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
           <t>p18</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>p19</t>
-        </is>
-      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>361-RC3210-S-01-BE022</t>
@@ -17934,12 +17932,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -17992,16 +17990,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Below</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>9</v>
+          <t>Above</t>
+        </is>
       </c>
       <c r="D22" t="n">
-        <v>440</v>
-      </c>
-      <c r="E22" t="inlineStr"/>
+        <v>438.9</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>PL10mm</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>BE023</t>
@@ -18009,7 +18008,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>p43</t>
+          <t>p200</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -18024,7 +18023,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -18054,7 +18053,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -18100,7 +18099,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>140</v>
+        <v>438.9</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -18181,7 +18180,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -18243,14 +18242,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>6</v>
       </c>
       <c r="D27" t="n">
-        <v>150</v>
+        <v>232</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
@@ -18260,7 +18259,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>p83</t>
+          <t>p33</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -18292,7 +18291,7 @@
         <v>6</v>
       </c>
       <c r="D28" t="n">
-        <v>232</v>
+        <v>150</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
@@ -18396,7 +18395,7 @@
         <v>7</v>
       </c>
       <c r="D30" t="n">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
@@ -18406,7 +18405,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>p101</t>
+          <t>p47</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -18473,14 +18472,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>7</v>
       </c>
       <c r="D32" t="n">
-        <v>115</v>
+        <v>90.5</v>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
@@ -18490,7 +18489,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>p101</t>
+          <t>p126</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -18519,10 +18518,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D33" t="n">
-        <v>60</v>
+        <v>115</v>
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
@@ -18532,7 +18531,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>p126</t>
+          <t>p125</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -18599,14 +18598,14 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D35" t="n">
-        <v>313</v>
+        <v>115</v>
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
@@ -18616,7 +18615,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>p100</t>
+          <t>p125</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -18641,7 +18640,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -18658,7 +18657,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>p124</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -18683,7 +18682,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -18695,7 +18694,7 @@
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>CO007</t>
+          <t>p100</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -18710,12 +18709,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -18732,7 +18731,7 @@
         <v>7</v>
       </c>
       <c r="D38" t="n">
-        <v>115</v>
+        <v>250</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
@@ -18742,7 +18741,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>p101</t>
+          <t>p92</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -18787,24 +18786,24 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C39" t="n">
         <v>7</v>
       </c>
       <c r="D39" t="n">
-        <v>90.5</v>
+        <v>250</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>p102</t>
+          <t>CO008</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>p126</t>
+          <t>p92</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -18814,12 +18813,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -18846,7 +18845,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>p125</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -18874,22 +18873,21 @@
           <t>Above</t>
         </is>
       </c>
+      <c r="C41" t="n">
+        <v>7</v>
+      </c>
       <c r="D41" t="n">
-        <v>116</v>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>PL9mm</t>
-        </is>
-      </c>
+        <v>90.5</v>
+      </c>
+      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>CO008</t>
+          <t>p102</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>p124</t>
+          <t>p126</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -18899,12 +18897,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -18921,7 +18919,7 @@
         <v>7</v>
       </c>
       <c r="D42" t="n">
-        <v>90.5</v>
+        <v>220</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
@@ -18931,7 +18929,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>p127</t>
+          <t>p125</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -18959,13 +18957,14 @@
           <t>Above</t>
         </is>
       </c>
-      <c r="C43" t="n">
-        <v>7</v>
-      </c>
       <c r="D43" t="n">
-        <v>60</v>
-      </c>
-      <c r="E43" t="inlineStr"/>
+        <v>220</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>PL9mm</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>CO008</t>
@@ -18973,7 +18972,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>p127</t>
+          <t>p124</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -18988,7 +18987,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -18998,24 +18997,25 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Below</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>7</v>
+          <t>Above</t>
+        </is>
       </c>
       <c r="D44" t="n">
-        <v>90</v>
-      </c>
-      <c r="E44" t="inlineStr"/>
+        <v>116</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>PL9mm</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>p101</t>
+          <t>CO008</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>p102</t>
+          <t>p124</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -19025,12 +19025,12 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -19040,19 +19040,19 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C45" t="n">
         <v>7</v>
       </c>
       <c r="D45" t="n">
-        <v>90.5</v>
+        <v>60</v>
       </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>p102</t>
+          <t>CO008</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -19067,12 +19067,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -19190,20 +19190,20 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D48" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>p15</t>
+          <t>CO009</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>p16</t>
+          <t>p17</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -19213,12 +19213,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -19228,24 +19228,24 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D49" t="n">
-        <v>158</v>
+        <v>343</v>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>p15</t>
+          <t>CO009</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>p7</t>
+          <t>p143</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -19255,12 +19255,12 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -19316,10 +19316,10 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D51" t="n">
-        <v>164.5</v>
+        <v>308</v>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
@@ -19329,7 +19329,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>p144</t>
+          <t>p7</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -19358,20 +19358,20 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="D52" t="n">
-        <v>400</v>
+        <v>197</v>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>p16</t>
+          <t>p143</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>p7</t>
+          <t>p144</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -19461,13 +19461,14 @@
           <t>Above</t>
         </is>
       </c>
-      <c r="C54" t="n">
-        <v>10</v>
-      </c>
       <c r="D54" t="n">
-        <v>262</v>
-      </c>
-      <c r="E54" t="inlineStr"/>
+        <v>139</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>PL12mm</t>
+        </is>
+      </c>
       <c r="F54" t="inlineStr">
         <is>
           <t>CO010</t>
@@ -19475,7 +19476,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>p169</t>
+          <t>p198</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -19490,7 +19491,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -19507,7 +19508,7 @@
         <v>10</v>
       </c>
       <c r="D55" t="n">
-        <v>262</v>
+        <v>350</v>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
@@ -19549,7 +19550,7 @@
         <v>9</v>
       </c>
       <c r="D56" t="n">
-        <v>139</v>
+        <v>260</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
@@ -19559,7 +19560,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>p184</t>
+          <t>p185</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -19584,11 +19585,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D57" t="n">
         <v>139</v>
@@ -19601,7 +19602,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>p185</t>
+          <t>p194</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -19626,14 +19627,14 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C58" t="n">
         <v>12</v>
       </c>
       <c r="D58" t="n">
-        <v>139</v>
+        <v>110</v>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
@@ -19643,7 +19644,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>p194</t>
+          <t>p197</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -19668,11 +19669,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D59" t="n">
         <v>139</v>
@@ -19685,7 +19686,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>p196</t>
+          <t>p197</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -19713,13 +19714,14 @@
           <t>Above</t>
         </is>
       </c>
-      <c r="C60" t="n">
-        <v>12</v>
-      </c>
       <c r="D60" t="n">
-        <v>110</v>
-      </c>
-      <c r="E60" t="inlineStr"/>
+        <v>260</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>PL12mm</t>
+        </is>
+      </c>
       <c r="F60" t="inlineStr">
         <is>
           <t>CO010</t>
@@ -19727,7 +19729,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>p197</t>
+          <t>p198</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -19742,7 +19744,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -19752,14 +19754,14 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D61" t="n">
-        <v>110</v>
+        <v>139</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
@@ -19769,7 +19771,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>p197</t>
+          <t>p199</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -19794,11 +19796,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D62" t="n">
         <v>139</v>
@@ -19811,7 +19813,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>p197</t>
+          <t>p199</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -19839,14 +19841,13 @@
           <t>Above</t>
         </is>
       </c>
+      <c r="C63" t="n">
+        <v>7</v>
+      </c>
       <c r="D63" t="n">
         <v>260</v>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>PL12mm</t>
-        </is>
-      </c>
+      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>CO010</t>
@@ -19854,7 +19855,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>p198</t>
+          <t>p199</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -19869,7 +19870,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -19886,7 +19887,7 @@
         <v>7</v>
       </c>
       <c r="D64" t="n">
-        <v>139</v>
+        <v>260</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
@@ -19928,7 +19929,7 @@
         <v>7</v>
       </c>
       <c r="D65" t="n">
-        <v>139</v>
+        <v>260</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
@@ -19963,14 +19964,14 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D66" t="n">
-        <v>260</v>
+        <v>139</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
@@ -19980,7 +19981,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>p199</t>
+          <t>p202</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -20005,14 +20006,14 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D67" t="n">
-        <v>260</v>
+        <v>139</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
@@ -20022,7 +20023,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>p199</t>
+          <t>p207</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -20051,7 +20052,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D68" t="n">
         <v>139</v>
@@ -20064,7 +20065,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>p202</t>
+          <t>p207</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -20089,14 +20090,14 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C69" t="n">
         <v>9</v>
       </c>
       <c r="D69" t="n">
-        <v>139</v>
+        <v>260</v>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
@@ -20135,10 +20136,10 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D70" t="n">
-        <v>260</v>
+        <v>139</v>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
@@ -20148,7 +20149,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>p207</t>
+          <t>p212</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -20222,17 +20223,17 @@
         <v>12</v>
       </c>
       <c r="D72" t="n">
-        <v>90</v>
+        <v>139</v>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>sp23</t>
+          <t>CO010</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>p183</t>
+          <t>p212</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -20242,12 +20243,12 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -20257,7 +20258,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -20311,7 +20312,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>p182</t>
+          <t>sp23</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -20353,7 +20354,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>p182</t>
+          <t>sp23</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -20395,7 +20396,7 @@
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>p182</t>
+          <t>sp23</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -20425,7 +20426,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -20509,26 +20510,27 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Below</t>
-        </is>
-      </c>
-      <c r="C79" t="n">
-        <v>12</v>
+          <t>Above</t>
+        </is>
       </c>
       <c r="D79" t="n">
-        <v>90</v>
-      </c>
-      <c r="E79" t="inlineStr"/>
+        <v>330</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>PL20mm</t>
+        </is>
+      </c>
       <c r="F79" t="inlineStr">
         <is>
+          <t>sp23</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
           <t>p182</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>p183</t>
-        </is>
-      </c>
       <c r="H79" t="inlineStr">
         <is>
           <t>361-RC3210-S-01-CO010</t>
@@ -20541,7 +20543,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -20554,13 +20556,14 @@
           <t>Above</t>
         </is>
       </c>
-      <c r="C80" t="n">
-        <v>9</v>
-      </c>
       <c r="D80" t="n">
-        <v>110</v>
-      </c>
-      <c r="E80" t="inlineStr"/>
+        <v>324</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>PL10mm</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr">
         <is>
           <t>p195</t>
@@ -20568,7 +20571,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>p196</t>
+          <t>p197</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -20583,7 +20586,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -20596,13 +20599,14 @@
           <t>Above</t>
         </is>
       </c>
-      <c r="C81" t="n">
-        <v>12</v>
-      </c>
       <c r="D81" t="n">
         <v>110</v>
       </c>
-      <c r="E81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>PL10mm</t>
+        </is>
+      </c>
       <c r="F81" t="inlineStr">
         <is>
           <t>p195</t>
@@ -20610,7 +20614,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>p212</t>
+          <t>p202</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -20625,7 +20629,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -20635,11 +20639,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D82" t="n">
         <v>110</v>
@@ -20652,7 +20656,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>p212</t>
+          <t>p196</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -20681,7 +20685,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D83" t="n">
         <v>110</v>
@@ -20694,7 +20698,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>p212</t>
+          <t>p196</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">

</xml_diff>

<commit_message>
Tighten leader angles to +/-10 deg from axes; refresh README and clean junk.
Ban near-horizontal/vertical diagonals (10-80 deg band), strengthen dense-cluster uncrossing, update docs, and remove one-off debug scripts, plot dumps, backups, and tracked annotated PDFs/Excel locks.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/焊缝统计_auto.xlsx
+++ b/焊缝统计_auto.xlsx
@@ -10630,19 +10630,19 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>461</v>
+        <v>140</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>BE018</t>
+          <t>p52</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -10657,12 +10657,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -10692,14 +10692,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>461</v>
+        <v>140</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
@@ -10709,7 +10709,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>p53</t>
+          <t>p52</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -10776,7 +10776,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -10838,24 +10838,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>220</v>
+        <v>140</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>BE019</t>
+          <t>p176</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>p118</t>
+          <t>p52</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -10865,12 +10865,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
         <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>220</v>
+        <v>140</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
@@ -10897,7 +10897,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>p118</t>
+          <t>p52</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -10922,14 +10922,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>12</v>
       </c>
       <c r="D8" t="n">
-        <v>300</v>
+        <v>445</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
@@ -10939,7 +10939,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>p118</t>
+          <t>p175</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -10984,7 +10984,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -10996,7 +10996,7 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>BE020</t>
+          <t>p175</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -11011,12 +11011,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -11026,14 +11026,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>7</v>
       </c>
       <c r="D10" t="n">
-        <v>39</v>
+        <v>140</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
@@ -11068,7 +11068,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -11080,7 +11080,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>BE020</t>
+          <t>p175</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -11095,12 +11095,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -11218,10 +11218,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D14" t="n">
-        <v>155</v>
+        <v>250</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>p123</t>
+          <t>p122</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -11263,12 +11263,12 @@
         <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>60</v>
+        <v>155</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>p122</t>
+          <t>BE021</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -11283,12 +11283,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -11305,12 +11305,12 @@
         <v>8</v>
       </c>
       <c r="D16" t="n">
-        <v>60</v>
+        <v>155</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>p122</t>
+          <t>BE021</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -11325,12 +11325,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -11340,16 +11340,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Below</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>12</v>
+          <t>Above</t>
+        </is>
       </c>
       <c r="D17" t="n">
-        <v>533.9</v>
-      </c>
-      <c r="E17" t="inlineStr"/>
+        <v>140</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PL10mm</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>BE022</t>
@@ -11357,7 +11358,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>p19</t>
+          <t>p200</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -11372,7 +11373,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -11405,14 +11406,13 @@
           <t>Above</t>
         </is>
       </c>
+      <c r="C18" t="n">
+        <v>6</v>
+      </c>
       <c r="D18" t="n">
-        <v>140</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>PL10mm</t>
-        </is>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>BE022</t>
@@ -11420,7 +11420,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>p200</t>
+          <t>p26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -11435,7 +11435,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -11487,7 +11487,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -11532,14 +11532,13 @@
           <t>Above</t>
         </is>
       </c>
+      <c r="C21" t="n">
+        <v>7</v>
+      </c>
       <c r="D21" t="n">
-        <v>438.9</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>PL10mm</t>
-        </is>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>BE022</t>
@@ -11547,7 +11546,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>p200</t>
+          <t>p18</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -11562,7 +11561,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>CJP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -11572,7 +11571,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -11634,14 +11633,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>440</v>
+        <v>140</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
@@ -11651,7 +11650,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>p43</t>
+          <t>p48</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -11722,13 +11721,14 @@
           <t>Above</t>
         </is>
       </c>
-      <c r="C25" t="n">
-        <v>6</v>
-      </c>
       <c r="D25" t="n">
-        <v>140</v>
-      </c>
-      <c r="E25" t="inlineStr"/>
+        <v>438.9</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>PL10mm</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>BE023</t>
@@ -11736,7 +11736,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>p48</t>
+          <t>p200</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -11823,7 +11823,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -11840,7 +11840,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>p83</t>
+          <t>p33</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -11865,14 +11865,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C28" t="n">
         <v>6</v>
       </c>
       <c r="D28" t="n">
-        <v>150</v>
+        <v>232</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
@@ -11907,14 +11907,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>7</v>
       </c>
       <c r="D29" t="n">
-        <v>115</v>
+        <v>250</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
@@ -11924,7 +11924,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>p101</t>
+          <t>p47</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -11969,14 +11969,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C30" t="n">
         <v>7</v>
       </c>
       <c r="D30" t="n">
-        <v>90.5</v>
+        <v>115</v>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
@@ -11986,7 +11986,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>p126</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -12018,7 +12018,7 @@
         <v>7</v>
       </c>
       <c r="D31" t="n">
-        <v>60</v>
+        <v>115</v>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
@@ -12028,7 +12028,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>p126</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -12060,17 +12060,17 @@
         <v>7</v>
       </c>
       <c r="D32" t="n">
-        <v>90.5</v>
+        <v>115</v>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>p100</t>
+          <t>CO007</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>p126</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -12080,12 +12080,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -12099,10 +12099,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D33" t="n">
-        <v>115</v>
+        <v>220</v>
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
@@ -12137,16 +12137,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Below</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>9</v>
+          <t>Above</t>
+        </is>
       </c>
       <c r="D34" t="n">
-        <v>115</v>
-      </c>
-      <c r="E34" t="inlineStr"/>
+        <v>116</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>PL9mm</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr">
         <is>
           <t>CO007</t>
@@ -12154,7 +12155,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>p125</t>
+          <t>p124</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -12169,7 +12170,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -12225,21 +12226,22 @@
           <t>Above</t>
         </is>
       </c>
-      <c r="C36" t="n">
-        <v>7</v>
-      </c>
       <c r="D36" t="n">
-        <v>90.5</v>
-      </c>
-      <c r="E36" t="inlineStr"/>
+        <v>116</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>PL9mm</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>p100</t>
+          <t>CO007</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>p101</t>
+          <t>p124</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -12249,12 +12251,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -12264,7 +12266,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -12276,12 +12278,12 @@
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>p100</t>
+          <t>CO007</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>p124</t>
+          <t>p127</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -12291,12 +12293,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -12313,7 +12315,7 @@
         <v>7</v>
       </c>
       <c r="D38" t="n">
-        <v>308</v>
+        <v>220</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
@@ -12323,7 +12325,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>p102</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -12368,14 +12370,14 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C39" t="n">
         <v>7</v>
       </c>
       <c r="D39" t="n">
-        <v>172</v>
+        <v>90.5</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
@@ -12385,7 +12387,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>p92</t>
+          <t>p126</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -12417,7 +12419,7 @@
         <v>7</v>
       </c>
       <c r="D40" t="n">
-        <v>115</v>
+        <v>90.5</v>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
@@ -12427,7 +12429,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>p101</t>
+          <t>p126</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -12459,7 +12461,7 @@
         <v>7</v>
       </c>
       <c r="D41" t="n">
-        <v>115</v>
+        <v>220</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
@@ -12469,7 +12471,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>p101</t>
+          <t>p125</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -12498,20 +12500,20 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D42" t="n">
-        <v>90.5</v>
+        <v>115</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>p102</t>
+          <t>CO008</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>p126</t>
+          <t>p125</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -12521,12 +12523,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -12539,13 +12541,14 @@
           <t>Above</t>
         </is>
       </c>
-      <c r="C43" t="n">
-        <v>7</v>
-      </c>
       <c r="D43" t="n">
-        <v>220</v>
-      </c>
-      <c r="E43" t="inlineStr"/>
+        <v>116</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>PL9mm</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>CO008</t>
@@ -12553,7 +12556,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>p125</t>
+          <t>p124</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -12568,7 +12571,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -12578,16 +12581,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Below</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>7</v>
+          <t>Above</t>
+        </is>
       </c>
       <c r="D44" t="n">
-        <v>220</v>
-      </c>
-      <c r="E44" t="inlineStr"/>
+        <v>116</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>PL9mm</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>CO008</t>
@@ -12595,7 +12599,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>p125</t>
+          <t>p124</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -12610,7 +12614,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>CJP</t>
         </is>
       </c>
     </row>
@@ -12663,24 +12667,24 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C46" t="n">
         <v>7</v>
       </c>
       <c r="D46" t="n">
-        <v>90.5</v>
+        <v>90</v>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>CO008</t>
+          <t>p101</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>p127</t>
+          <t>p102</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -12690,12 +12694,12 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>
@@ -12712,7 +12716,7 @@
         <v>16</v>
       </c>
       <c r="D47" t="n">
-        <v>158</v>
+        <v>120</v>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
@@ -12722,7 +12726,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>p7</t>
+          <t>p16</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -12767,24 +12771,24 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Above</t>
+          <t>Below</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D48" t="n">
-        <v>158</v>
+        <v>38</v>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>p15</t>
+          <t>CO009</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>p7</t>
+          <t>p17</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -12794,12 +12798,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>LJ</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>PP</t>
+          <t>FW</t>
         </is>
       </c>
     </row>
@@ -12851,14 +12855,14 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Below</t>
+          <t>Above</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D50" t="n">
-        <v>343</v>
+        <v>405</v>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
@@ -12868,7 +12872,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>p143</t>
+          <t>p7</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -12900,7 +12904,7 @@
         <v>16</v>
       </c>
       <c r="D51" t="n">
-        <v>308</v>
+        <v>405</v>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
@@ -12942,12 +12946,12 @@
         <v>7</v>
       </c>
       <c r="D52" t="n">
-        <v>164.5</v>
+        <v>197</v>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>CO009</t>
+          <t>p143</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -12962,12 +12966,12 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>LJ</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>PP</t>
         </is>
       </c>
     </row>

</xml_diff>